<commit_message>
Update service request tests, add keywords, docs, and utility scripts
</commit_message>
<xml_diff>
--- a/data/commercial_loan_extension.xlsx
+++ b/data/commercial_loan_extension.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="LoanExtension" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,44 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +70,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,24 +459,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Customer ID</t>
-        </is>
-      </c>
+      <c r="A1" s="1">
+        <f>== STANDARD SECTION ===</f>
+        <v/>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Customer ID</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Reschedulement_Type</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>New_Tenure</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>New_Installment_Amount</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Borrower_Status</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Service_Charges_Waiver</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Payment_Mode</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>200125</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tenure</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Non Default</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Cash-Cheque</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Standard loan extension</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <f>== BALLOON SECTION ===</f>
+        <v/>
+      </c>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Balloon_Type</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Balloon_Frequency</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Balloon_Amount</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Balloon_Installments</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Balloon</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>QUARTERLY</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Tenure,Installment"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Default,Non Default"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"KNet-Kiosk,KNet-Web,Cash-Cheque"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Balloon,Regular EMI"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"MONTHLY,QUARTERLY,Half Yearly,Yearly"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>